<commit_message>
Add legal pages, security hardening, and Hudak restyle
</commit_message>
<xml_diff>
--- a/Hudak/hudak_sablon.xlsx
+++ b/Hudak/hudak_sablon.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zsomborgalgoczi/Desktop/label labor assets/label_generator_excels/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zsomborgalgoczi/Desktop/workspace/github.com/zsombzs/label_generator/Hudak/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03AD74F0-11B9-6E43-8216-D88F8EF629CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E008120-0DDF-B74E-8C30-C0CAEB166C3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16960" xr2:uid="{195B7CB8-57D0-714D-A057-F87136F4FC09}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Cikkszám</t>
   </si>
@@ -51,6 +51,9 @@
   </si>
   <si>
     <t>Ár</t>
+  </si>
+  <si>
+    <t>Akciós_ár</t>
   </si>
 </sst>
 </file>
@@ -87,7 +90,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -154,11 +157,22 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thick">
+        <color auto="1"/>
+      </left>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -177,6 +191,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -511,7 +526,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0807640-E514-5C42-8365-97613778117F}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35.1640625" style="7" customWidth="1"/>
@@ -519,9 +534,10 @@
     <col min="3" max="3" width="33.33203125" customWidth="1"/>
     <col min="4" max="4" width="27.33203125" customWidth="1"/>
     <col min="5" max="5" width="29" style="5" customWidth="1"/>
+    <col min="6" max="6" width="23.33203125" style="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="43" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="43" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -537,8 +553,11 @@
       <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
     </row>
-    <row r="2" spans="1:5" ht="17" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A2" s="6"/>
       <c r="B2" s="4"/>
     </row>

</xml_diff>